<commit_message>
HW03 submission: add reports, screenshots, fixes
Add full HW03 submission artifacts and adjust notes: added screenshots and evidence (multiple PNGs), LinkQuayScreenRecording.txt, ai_audit.md/pdf, ai_critique.pdf, and bug_reports_gui.md. Updated participant session notes P02–P07, findings-report.md (timings and finding details), and test-plan.md (participant P05). Updated gui_checklist.xlsx and test-plan metadata. These changes consolidate GUI test evidence, AI audit records, and correct several observed test details.
</commit_message>
<xml_diff>
--- a/HW03-submission/gui_checklist.xlsx
+++ b/HW03-submission/gui_checklist.xlsx
@@ -8,19 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA_D\ProjectGitHub\Group06_HW2_Testing\HW03-submission\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BA02AB-059C-4862-A999-23828DFDBCFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4C546B-3446-4418-BFD2-A9ED8220F3B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2798" yWindow="1882" windowWidth="16199" windowHeight="9848" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GUI Checklist" sheetId="1" r:id="rId1"/>
+    <sheet name="Cross_Browser_Matrix" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cross_Browser_Matrix!$A$3:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GUI Checklist'!$F$2:$F$46</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="225">
   <si>
     <t>ID</t>
   </si>
@@ -403,6 +408,9 @@
     <t>Trình duyệt gợi ý tự động đúng trường (name, tel, street-address)</t>
   </si>
   <si>
+    <t>Profile có các input (name, phone, address) KHÔNG có thuộc tính autocomplete. Trình duyệt không gợi ý tự động.</t>
+  </si>
+  <si>
     <t>GUI-28</t>
   </si>
   <si>
@@ -412,6 +420,9 @@
     <t>Input SĐT có type=tel để mobile hiện numeric keyboard (FR-04, FR-22)</t>
   </si>
   <si>
+    <t>Profile dùn input Số điện thoại dùng type=text thay vì type=tel.Vi phạm FR-04.</t>
+  </si>
+  <si>
     <t>GUI-29</t>
   </si>
   <si>
@@ -655,10 +666,40 @@
     <t>Màu Primary (nút hành động tích cực) KHÔNG NHẤT QUÁN. FR-21 yêu cầu Primary = xanh dương. ProductDetail/Cart/Checkout/Register dùng green/red.</t>
   </si>
   <si>
-    <t>Profile có các input (name, phone, address) KHÔNG có thuộc tính autocomplete. Trình duyệt không gợi ý tự động.</t>
-  </si>
-  <si>
-    <t>Profile dùn input Số điện thoại dùng type=text thay vì type=tel.Vi phạm FR-04.</t>
+    <t>Cross-Browser Test Matrix - GUI Checklist</t>
+  </si>
+  <si>
+    <t>Thông tin Item</t>
+  </si>
+  <si>
+    <t>Kết quả kiểm tra trên trình duyệt / nền tảng (Passed / Failed / N/A)</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
+  </si>
+  <si>
+    <t>Item ID</t>
+  </si>
+  <si>
+    <t>Interface Aspect</t>
+  </si>
+  <si>
+    <t>Checklist Description</t>
+  </si>
+  <si>
+    <t>Chrome (Desktop)</t>
+  </si>
+  <si>
+    <t>Firefox (Desktop)</t>
+  </si>
+  <si>
+    <t>Edge (Desktop)</t>
+  </si>
+  <si>
+    <t>Cross-Browser Issues / Notes</t>
+  </si>
+  <si>
+    <t>Kết quả kiểm tra nhất quán 100% trên cả 4 trình duyệt (Chrome, Edge, Cốc Cốc, Firefox). Không phát hiện lỗi sai lệch hiển thị (Layout inconsistency) hay lỗi tương thích cross-browser.</t>
   </si>
 </sst>
 </file>
@@ -699,7 +740,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -730,8 +771,23 @@
         <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -739,11 +795,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -759,6 +830,28 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1062,6 +1155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1074,7 +1168,7 @@
     <col min="7" max="7" width="126.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1097,7 +1191,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1120,7 +1214,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -1143,7 +1237,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1166,7 +1260,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
@@ -1189,7 +1283,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1212,7 +1306,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -1235,7 +1329,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
@@ -1258,7 +1352,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
@@ -1281,7 +1375,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>44</v>
       </c>
@@ -1304,7 +1398,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>48</v>
       </c>
@@ -1327,7 +1421,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>52</v>
       </c>
@@ -1350,7 +1444,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>56</v>
       </c>
@@ -1373,7 +1467,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>61</v>
       </c>
@@ -1396,7 +1490,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>65</v>
       </c>
@@ -1419,7 +1513,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>69</v>
       </c>
@@ -1442,7 +1536,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>73</v>
       </c>
@@ -1465,7 +1559,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>78</v>
       </c>
@@ -1488,7 +1582,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>82</v>
       </c>
@@ -1511,7 +1605,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>86</v>
       </c>
@@ -1534,7 +1628,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>90</v>
       </c>
@@ -1557,7 +1651,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>95</v>
       </c>
@@ -1580,7 +1674,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>99</v>
       </c>
@@ -1603,7 +1697,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>105</v>
       </c>
@@ -1626,7 +1720,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>110</v>
       </c>
@@ -1649,7 +1743,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>114</v>
       </c>
@@ -1672,7 +1766,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>119</v>
       </c>
@@ -1695,7 +1789,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>123</v>
       </c>
@@ -1715,12 +1809,12 @@
         <v>12</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>124</v>
@@ -1729,410 +1823,1531 @@
         <v>101</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>101</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>101</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E31" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A32" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>101</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F33" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A34" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="D34" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F39" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A40" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="D40" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>57</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>74</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="30.75" x14ac:dyDescent="0.45">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>12</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="15.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="30.75" x14ac:dyDescent="0.45">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="F2:F46" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Failed"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="4" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+    </row>
+    <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A4" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A7" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A10" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A11" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A13" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A14" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A15" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A16" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A17" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A18" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A19" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A21" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A22" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A23" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A24" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A25" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A26" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A27" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A28" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A29" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A30" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A31" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A32" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A33" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A34" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A35" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A36" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A37" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A38" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A39" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A40" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A41" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A42" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A43" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A44" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A45" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A46" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A47" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A48" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:G48" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <mergeCells count="4">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="G2"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn: Passed, Failed, hoặc N/A" sqref="D4:F48" xr:uid="{00000000-0002-0000-0100-000000000000}">
+      <formula1>"Passed,Failed,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>